<commit_message>
Migration progress, additional pages + blocks
Automated migration updates generated by Experience Modernization Agent.

Changed files: 126
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article.report.xlsx
+++ b/tools/importer/reports/import-article.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="314">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,7 +58,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-03T05:59:39.568Z</t>
+    <t>2026-10-06T20:54:42.343Z</t>
   </si>
   <si>
     <t>Bradesco Bank</t>
@@ -67,6 +67,78 @@
     <t>https://bradescobank.com/</t>
   </si>
   <si>
+    <t>en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-feature"]</t>
+  </si>
+  <si>
+    <t>en/about-us</t>
+  </si>
+  <si>
+    <t>info-page</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:00:49.665Z</t>
+  </si>
+  <si>
+    <t>About us – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/about-us/</t>
+  </si>
+  <si>
+    <t>en/articles-archive.report.json</t>
+  </si>
+  <si>
+    <t>en/articles-archive</t>
+  </si>
+  <si>
+    <t>listing</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:06:22.399Z</t>
+  </si>
+  <si>
+    <t>Articles Archive – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/articles-archive/</t>
+  </si>
+  <si>
+    <t>en/bank-holidays.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","table-article"]</t>
+  </si>
+  <si>
+    <t>en/bank-holidays</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:02:08.338Z</t>
+  </si>
+  <si>
+    <t>Bank Holidays – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/bank-holidays/</t>
+  </si>
+  <si>
+    <t>en/bradesco-lounge.report.json</t>
+  </si>
+  <si>
+    <t>en/bradesco-lounge</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:02:20.222Z</t>
+  </si>
+  <si>
+    <t>Bradesco Lounge – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/bradesco-lounge/</t>
+  </si>
+  <si>
     <t>en/careers.report.json</t>
   </si>
   <si>
@@ -79,7 +151,7 @@
     <t>landing</t>
   </si>
   <si>
-    <t>2026-10-03T04:05:33.830Z</t>
+    <t>2026-10-06T20:00:11.724Z</t>
   </si>
   <si>
     <t>Careers – Bradesco Bank</t>
@@ -97,7 +169,7 @@
     <t>en/certificate-of-deposit-bradesco</t>
   </si>
   <si>
-    <t>2026-10-03T04:04:29.009Z</t>
+    <t>2026-10-06T19:59:17.095Z</t>
   </si>
   <si>
     <t>CDB – Bradesco Bank</t>
@@ -115,7 +187,7 @@
     <t>en/corporate</t>
   </si>
   <si>
-    <t>2026-10-03T04:02:38.500Z</t>
+    <t>2026-10-06T19:57:38.704Z</t>
   </si>
   <si>
     <t>Business Corporate – Bradesco Bank</t>
@@ -124,6 +196,21 @@
     <t>https://bradescobank.com/en/corporate/</t>
   </si>
   <si>
+    <t>en/cra-public-file.report.json</t>
+  </si>
+  <si>
+    <t>en/cra-public-file</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:01.832Z</t>
+  </si>
+  <si>
+    <t>CRA Public File – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/cra-public-file/</t>
+  </si>
+  <si>
     <t>en/credit-card-signature-gold.report.json</t>
   </si>
   <si>
@@ -133,7 +220,7 @@
     <t>en/credit-card-signature-gold</t>
   </si>
   <si>
-    <t>2026-10-03T04:04:15.702Z</t>
+    <t>2026-10-06T19:59:07.014Z</t>
   </si>
   <si>
     <t>Signature &amp; Gold – Bradesco Bank</t>
@@ -151,7 +238,7 @@
     <t>en/credit-cards</t>
   </si>
   <si>
-    <t>2026-10-03T04:03:54.970Z</t>
+    <t>2026-10-06T19:58:49.057Z</t>
   </si>
   <si>
     <t>Credit Cards – Bradesco Bank</t>
@@ -160,6 +247,27 @@
     <t>https://bradescobank.com/en/credit-cards/</t>
   </si>
   <si>
+    <t>en/exploring-investment-products-in-the-u-s.report.json</t>
+  </si>
+  <si>
+    <t>["hero-article","accordion"]</t>
+  </si>
+  <si>
+    <t>en/exploring-investment-products-in-the-u-s</t>
+  </si>
+  <si>
+    <t>article-rich</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:38.395Z</t>
+  </si>
+  <si>
+    <t>Exploring Investment Products in the U.S. – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/exploring-investment-products-in-the-u-s/</t>
+  </si>
+  <si>
     <t>en/financial-habits.report.json</t>
   </si>
   <si>
@@ -172,7 +280,7 @@
     <t>article</t>
   </si>
   <si>
-    <t>2026-10-03T05:59:49.901Z</t>
+    <t>2026-10-06T20:54:52.808Z</t>
   </si>
   <si>
     <t>Financial Habits – Bradesco Bank</t>
@@ -187,7 +295,7 @@
     <t>en/gold-as-a-portfolio-diversifier</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:00.829Z</t>
+    <t>2026-10-06T20:55:03.290Z</t>
   </si>
   <si>
     <t>Gold as a Portfolio Diversifier – Bradesco Bank</t>
@@ -196,6 +304,24 @@
     <t>https://bradescobank.com/en/gold-as-a-portfolio-diversifier/</t>
   </si>
   <si>
+    <t>en/help.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-media","cards-feature"]</t>
+  </si>
+  <si>
+    <t>en/help</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:01:58.243Z</t>
+  </si>
+  <si>
+    <t>How Can We Help? – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/help/</t>
+  </si>
+  <si>
     <t>en/how-to-buy-assets.report.json</t>
   </si>
   <si>
@@ -205,7 +331,7 @@
     <t>en/how-to-buy-assets</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:11.610Z</t>
+    <t>2026-10-06T20:55:14.991Z</t>
   </si>
   <si>
     <t>How to buy assets – Bradesco Bank</t>
@@ -220,7 +346,7 @@
     <t>en/how-to-sell-assets</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:20.362Z</t>
+    <t>2026-10-06T20:55:24.319Z</t>
   </si>
   <si>
     <t>How to sell assets – Bradesco Bank</t>
@@ -229,13 +355,64 @@
     <t>https://bradescobank.com/en/how-to-sell-assets/</t>
   </si>
   <si>
+    <t>en/insights-archive.report.json</t>
+  </si>
+  <si>
+    <t>en/insights-archive</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:06:41.844Z</t>
+  </si>
+  <si>
+    <t>Insights Archive – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/insights-archive/</t>
+  </si>
+  <si>
+    <t>en/institutional.report.json</t>
+  </si>
+  <si>
+    <t>["hero-video","hero-promo","columns-media","cards-feature","cards-feature"]</t>
+  </si>
+  <si>
+    <t>en/institutional</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:01:47.292Z</t>
+  </si>
+  <si>
+    <t>Business – Institutional – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/institutional/</t>
+  </si>
+  <si>
+    <t>en/investing-for-different-client-profiles.report.json</t>
+  </si>
+  <si>
+    <t>["hero-article","cards-feature","cards-feature"]</t>
+  </si>
+  <si>
+    <t>en/investing-for-different-client-profiles</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:52.992Z</t>
+  </si>
+  <si>
+    <t>Investing for Different Client Profiles – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/investing-for-different-client-profiles/</t>
+  </si>
+  <si>
     <t>en/investments-at-bradesco-bank.report.json</t>
   </si>
   <si>
     <t>en/investments-at-bradesco-bank</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:29.530Z</t>
+    <t>2026-10-06T20:55:34.037Z</t>
   </si>
   <si>
     <t>The Impact of Human Behavior on Financial Markets: Insights for Investors – Bradesco Bank</t>
@@ -244,13 +421,31 @@
     <t>https://bradescobank.com/en/investments-at-bradesco-bank/</t>
   </si>
   <si>
+    <t>en/investments-content.report.json</t>
+  </si>
+  <si>
+    <t>["hero-video","cards-feature","cards-feature","cards-audience"]</t>
+  </si>
+  <si>
+    <t>en/investments-content</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:06:00.724Z</t>
+  </si>
+  <si>
+    <t>Investments Content – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/investments-content/</t>
+  </si>
+  <si>
     <t>en/mutual-funds.report.json</t>
   </si>
   <si>
     <t>en/mutual-funds</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:39.281Z</t>
+    <t>2026-10-06T20:55:44.848Z</t>
   </si>
   <si>
     <t>Mutual Funds – Bradesco Bank</t>
@@ -265,7 +460,7 @@
     <t>en/open-an-investment-account</t>
   </si>
   <si>
-    <t>2026-10-03T06:00:49.886Z</t>
+    <t>2026-10-06T20:55:56.566Z</t>
   </si>
   <si>
     <t>Open an investment account – Bradesco Bank</t>
@@ -274,6 +469,21 @@
     <t>https://bradescobank.com/en/open-an-investment-account/</t>
   </si>
   <si>
+    <t>en/other-disclosures.report.json</t>
+  </si>
+  <si>
+    <t>en/other-disclosures</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:02:51.750Z</t>
+  </si>
+  <si>
+    <t>Other disclosures – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/other-disclosures/</t>
+  </si>
+  <si>
     <t>en/personal-bank.report.json</t>
   </si>
   <si>
@@ -283,7 +493,7 @@
     <t>en/personal-bank</t>
   </si>
   <si>
-    <t>2026-10-03T04:00:39.590Z</t>
+    <t>2026-10-06T19:57:09.911Z</t>
   </si>
   <si>
     <t>Personal Bank – Bradesco Bank</t>
@@ -298,7 +508,7 @@
     <t>en/portfolio-considerations-the-role-of-staying-invested</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:00.728Z</t>
+    <t>2026-10-06T20:56:05.589Z</t>
   </si>
   <si>
     <t>Portfolio Considerations: The role of staying invested – Bradesco Bank</t>
@@ -307,6 +517,24 @@
     <t>https://bradescobank.com/en/portfolio-considerations-the-role-of-staying-invested/</t>
   </si>
   <si>
+    <t>en/privacy-and-cookies.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","table-article","table-article","table-article","table-article","table-article","table-article","table-article","table-article","table-article","tabs"]</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:02:41.572Z</t>
+  </si>
+  <si>
+    <t>Privacy and Cookies – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/</t>
+  </si>
+  <si>
     <t>en/private-bank.report.json</t>
   </si>
   <si>
@@ -316,7 +544,7 @@
     <t>en/private-bank</t>
   </si>
   <si>
-    <t>2026-10-03T04:01:38.279Z</t>
+    <t>2026-10-06T19:57:25.389Z</t>
   </si>
   <si>
     <t>Private Bank – Bradesco Bank</t>
@@ -334,7 +562,7 @@
     <t>en/real-estate</t>
   </si>
   <si>
-    <t>2026-10-03T04:03:38.801Z</t>
+    <t>2026-10-06T19:58:36.763Z</t>
   </si>
   <si>
     <t>Real Estate – Bradesco Bank</t>
@@ -352,7 +580,7 @@
     <t>en/reits</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:11.826Z</t>
+    <t>2026-10-06T20:56:15.637Z</t>
   </si>
   <si>
     <t>REITs – Bradesco Bank</t>
@@ -361,13 +589,49 @@
     <t>https://bradescobank.com/en/reits/</t>
   </si>
   <si>
+    <t>en/security.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-media","cards-feature","cards-feature","accordion"]</t>
+  </si>
+  <si>
+    <t>en/security</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:02:30.211Z</t>
+  </si>
+  <si>
+    <t>Security – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/security/</t>
+  </si>
+  <si>
+    <t>en/the-power-of-compounding.report.json</t>
+  </si>
+  <si>
+    <t>["hero-article","cards-feature","cards-feature","table-article","compound-calculator"]</t>
+  </si>
+  <si>
+    <t>en/the-power-of-compounding</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:04:02.964Z</t>
+  </si>
+  <si>
+    <t>The Power of Compounding – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/the-power-of-compounding/</t>
+  </si>
+  <si>
     <t>en/thematic-etfs.report.json</t>
   </si>
   <si>
     <t>en/thematic-etfs</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:22.594Z</t>
+    <t>2026-10-06T20:56:25.801Z</t>
   </si>
   <si>
     <t>Thematic ETFs – Bradesco Bank</t>
@@ -382,7 +646,7 @@
     <t>en/u-s-stocks</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:34.129Z</t>
+    <t>2026-10-06T20:56:36.091Z</t>
   </si>
   <si>
     <t>U.S. Stocks – Bradesco Bank</t>
@@ -397,7 +661,7 @@
     <t>en/what-are-asset-allocation-and-diversification</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:44.631Z</t>
+    <t>2026-10-06T20:56:46.213Z</t>
   </si>
   <si>
     <t>What Are Asset Allocation and Diversification? – Bradesco Bank</t>
@@ -412,7 +676,7 @@
     <t>en/why-invest-abroad</t>
   </si>
   <si>
-    <t>2026-10-03T06:01:55.055Z</t>
+    <t>2026-10-06T20:56:55.794Z</t>
   </si>
   <si>
     <t>Why Invest Abroad? – Bradesco Bank</t>
@@ -430,7 +694,7 @@
     <t>en/zelle</t>
   </si>
   <si>
-    <t>2026-10-03T04:04:40.830Z</t>
+    <t>2026-10-06T19:59:28.063Z</t>
   </si>
   <si>
     <t>Zelle – Bradesco Bank</t>
@@ -448,7 +712,7 @@
     <t>en/credit-card/visa-infinite</t>
   </si>
   <si>
-    <t>2026-10-03T04:04:54.933Z</t>
+    <t>2026-10-06T19:59:39.150Z</t>
   </si>
   <si>
     <t>Visa Infinite – Bradesco Bank</t>
@@ -466,7 +730,7 @@
     <t>en/investments-content/bradesco-investments-app</t>
   </si>
   <si>
-    <t>2026-10-03T04:05:22.845Z</t>
+    <t>2026-10-06T20:00:00.137Z</t>
   </si>
   <si>
     <t>Bradesco Investments App – Bradesco Bank</t>
@@ -475,6 +739,45 @@
     <t>https://bradescobank.com/en/investments-content/bradesco-investments-app/</t>
   </si>
   <si>
+    <t>en/investments-content/saved-articles.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner"]</t>
+  </si>
+  <si>
+    <t>en/investments-content/saved-articles</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:06:51.967Z</t>
+  </si>
+  <si>
+    <t>Saved Articles – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/investments-content/saved-articles/</t>
+  </si>
+  <si>
+    <t>en/personal-bank/faq.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","tabs"]</t>
+  </si>
+  <si>
+    <t>en/personal-bank/faq</t>
+  </si>
+  <si>
+    <t>faq-hub</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:04:51.315Z</t>
+  </si>
+  <si>
+    <t>FAQ – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/personal-bank/faq/</t>
+  </si>
+  <si>
     <t>en/personal-bank/investments.report.json</t>
   </si>
   <si>
@@ -484,7 +787,7 @@
     <t>en/personal-bank/investments</t>
   </si>
   <si>
-    <t>2026-10-03T04:05:08.962Z</t>
+    <t>2026-10-06T19:59:49.830Z</t>
   </si>
   <si>
     <t>Investments – Bradesco Bank</t>
@@ -505,7 +808,7 @@
     <t>en/careers/fragments/internship</t>
   </si>
   <si>
-    <t>2026-10-03T04:06:37.071Z</t>
+    <t>2026-10-06T20:00:37.937Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/careers/?fragment=internship</t>
@@ -523,10 +826,133 @@
     <t>en/careers/fragments/jobs</t>
   </si>
   <si>
-    <t>2026-10-03T04:06:24.633Z</t>
+    <t>2026-10-06T20:00:27.668Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/careers/?fragment=jobs</t>
+  </si>
+  <si>
+    <t>en/personal-bank/investments/faq.report.json</t>
+  </si>
+  <si>
+    <t>en/personal-bank/investments/faq</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:05:19.670Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/personal-bank/investments/faq/</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/bradesco-investments-privacy-notice.report.json</t>
+  </si>
+  <si>
+    <t>["table-article","table-article","table-article","table-article"]</t>
+  </si>
+  <si>
+    <t>bradesco-investments-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/bradesco-investments-privacy-notice</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:31.735Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=bradesco-investments-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/california-consumer-privacy-act-ccpa.report.json</t>
+  </si>
+  <si>
+    <t>["table-article"]</t>
+  </si>
+  <si>
+    <t>california-consumer-privacy-act-ccpa</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/california-consumer-privacy-act-ccpa</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:53.246Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=california-consumer-privacy-act-ccpa</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/childrens-privacy-policy.report.json</t>
+  </si>
+  <si>
+    <t>childrens-privacy-policy</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/childrens-privacy-policy</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:04:04.348Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=childrens-privacy-policy</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/consumer-privacy-notice.report.json</t>
+  </si>
+  <si>
+    <t>consumer-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/consumer-privacy-notice</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:17.517Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=consumer-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/online-privacy-notice.report.json</t>
+  </si>
+  <si>
+    <t>online-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/online-privacy-notice</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:03:41.991Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=online-privacy-notice</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/others.report.json</t>
+  </si>
+  <si>
+    <t>others</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/others</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:04:27.136Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=others</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/sms-terms-of-service.report.json</t>
+  </si>
+  <si>
+    <t>sms-terms-of-service</t>
+  </si>
+  <si>
+    <t>en/privacy-and-cookies/fragments/sms-terms-of-service</t>
+  </si>
+  <si>
+    <t>2026-10-06T20:04:16.131Z</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=sms-terms-of-service</t>
   </si>
 </sst>
 </file>
@@ -915,13 +1341,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
@@ -1018,19 +1444,19 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
         <v>27</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
       </c>
       <c r="G4" t="s">
         <v>28</v>
@@ -1076,13 +1502,13 @@
         <v>37</v>
       </c>
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
         <v>38</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
-        <v>39</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
@@ -1091,33 +1517,33 @@
         <v>21</v>
       </c>
       <c r="G6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
         <v>40</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>41</v>
-      </c>
-      <c r="I6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
         <v>44</v>
       </c>
-      <c r="C7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
         <v>45</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
-        <v>21</v>
       </c>
       <c r="G7" t="s">
         <v>46</v>
@@ -1146,24 +1572,24 @@
         <v>13</v>
       </c>
       <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
         <v>52</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>53</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>54</v>
-      </c>
-      <c r="I8" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
         <v>56</v>
-      </c>
-      <c r="B9" t="s">
-        <v>50</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -1175,7 +1601,7 @@
         <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
         <v>58</v>
@@ -1192,36 +1618,36 @@
         <v>61</v>
       </c>
       <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
         <v>62</v>
       </c>
-      <c r="C10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
         <v>63</v>
       </c>
-      <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>64</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>65</v>
-      </c>
-      <c r="I10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
         <v>67</v>
-      </c>
-      <c r="B11" t="s">
-        <v>62</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -1233,7 +1659,7 @@
         <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G11" t="s">
         <v>69</v>
@@ -1250,419 +1676,419 @@
         <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="G12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
       </c>
       <c r="F13" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I13" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E14" t="s">
         <v>13</v>
       </c>
       <c r="F14" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="G14" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I14" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
         <v>88</v>
       </c>
-      <c r="C15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" t="s">
-        <v>89</v>
-      </c>
-      <c r="E15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s">
-        <v>21</v>
-      </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H15" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I15" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
         <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
         <v>13</v>
       </c>
       <c r="F16" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="G16" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I16" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
       </c>
       <c r="F17" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="G17" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H17" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I17" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B18" t="s">
         <v>104</v>
       </c>
-      <c r="B18" t="s">
-        <v>105</v>
-      </c>
       <c r="C18" t="s">
         <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E18" t="s">
         <v>13</v>
       </c>
       <c r="F18" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="G18" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H18" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="I18" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="E19" t="s">
         <v>13</v>
       </c>
       <c r="F19" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="G19" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H19" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
         <v>11</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E20" t="s">
         <v>13</v>
       </c>
       <c r="F20" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H20" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I20" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>126</v>
       </c>
       <c r="C21" t="s">
         <v>11</v>
       </c>
       <c r="D21" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E21" t="s">
         <v>13</v>
       </c>
       <c r="F21" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="H21" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="I21" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E22" t="s">
         <v>13</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="G22" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="H22" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="I22" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>137</v>
       </c>
       <c r="C23" t="s">
         <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="E23" t="s">
         <v>13</v>
       </c>
       <c r="F23" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="G23" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="H23" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="I23" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B24" t="s">
-        <v>137</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
         <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E24" t="s">
         <v>13</v>
       </c>
       <c r="F24" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="G24" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H24" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="I24" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B25" t="s">
-        <v>143</v>
+        <v>104</v>
       </c>
       <c r="C25" t="s">
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E25" t="s">
         <v>13</v>
       </c>
       <c r="F25" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="G25" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="H25" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="I25" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B26" t="s">
-        <v>149</v>
+        <v>19</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E26" t="s">
         <v>13</v>
@@ -1671,85 +2097,85 @@
         <v>21</v>
       </c>
       <c r="G26" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H26" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I26" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B27" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E27" t="s">
         <v>13</v>
       </c>
       <c r="F27" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="G27" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H27" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="I27" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B28" t="s">
-        <v>161</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
-        <v>162</v>
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E28" t="s">
         <v>13</v>
       </c>
       <c r="F28" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="G28" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H28" t="s">
-        <v>23</v>
+        <v>166</v>
       </c>
       <c r="I28" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B29" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C29" t="s">
-        <v>168</v>
+        <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
@@ -1758,13 +2184,738 @@
         <v>21</v>
       </c>
       <c r="G29" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H29" t="s">
-        <v>23</v>
+        <v>172</v>
       </c>
       <c r="I29" t="s">
-        <v>171</v>
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>174</v>
+      </c>
+      <c r="B30" t="s">
+        <v>175</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="s">
+        <v>176</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
+        <v>45</v>
+      </c>
+      <c r="G30" t="s">
+        <v>177</v>
+      </c>
+      <c r="H30" t="s">
+        <v>178</v>
+      </c>
+      <c r="I30" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>180</v>
+      </c>
+      <c r="B31" t="s">
+        <v>181</v>
+      </c>
+      <c r="C31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" t="s">
+        <v>182</v>
+      </c>
+      <c r="E31" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" t="s">
+        <v>183</v>
+      </c>
+      <c r="H31" t="s">
+        <v>184</v>
+      </c>
+      <c r="I31" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" t="s">
+        <v>187</v>
+      </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" t="s">
+        <v>188</v>
+      </c>
+      <c r="E32" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" t="s">
+        <v>88</v>
+      </c>
+      <c r="G32" t="s">
+        <v>189</v>
+      </c>
+      <c r="H32" t="s">
+        <v>190</v>
+      </c>
+      <c r="I32" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>192</v>
+      </c>
+      <c r="B33" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" t="s">
+        <v>194</v>
+      </c>
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" t="s">
+        <v>195</v>
+      </c>
+      <c r="H33" t="s">
+        <v>196</v>
+      </c>
+      <c r="I33" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>198</v>
+      </c>
+      <c r="B34" t="s">
+        <v>199</v>
+      </c>
+      <c r="C34" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" t="s">
+        <v>200</v>
+      </c>
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
+        <v>81</v>
+      </c>
+      <c r="G34" t="s">
+        <v>201</v>
+      </c>
+      <c r="H34" t="s">
+        <v>202</v>
+      </c>
+      <c r="I34" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>204</v>
+      </c>
+      <c r="B35" t="s">
+        <v>86</v>
+      </c>
+      <c r="C35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" t="s">
+        <v>205</v>
+      </c>
+      <c r="E35" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
+        <v>88</v>
+      </c>
+      <c r="G35" t="s">
+        <v>206</v>
+      </c>
+      <c r="H35" t="s">
+        <v>207</v>
+      </c>
+      <c r="I35" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>209</v>
+      </c>
+      <c r="B36" t="s">
+        <v>86</v>
+      </c>
+      <c r="C36" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s">
+        <v>88</v>
+      </c>
+      <c r="G36" t="s">
+        <v>211</v>
+      </c>
+      <c r="H36" t="s">
+        <v>212</v>
+      </c>
+      <c r="I36" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>214</v>
+      </c>
+      <c r="B37" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" t="s">
+        <v>215</v>
+      </c>
+      <c r="E37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" t="s">
+        <v>88</v>
+      </c>
+      <c r="G37" t="s">
+        <v>216</v>
+      </c>
+      <c r="H37" t="s">
+        <v>217</v>
+      </c>
+      <c r="I37" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>219</v>
+      </c>
+      <c r="B38" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" t="s">
+        <v>220</v>
+      </c>
+      <c r="E38" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" t="s">
+        <v>88</v>
+      </c>
+      <c r="G38" t="s">
+        <v>221</v>
+      </c>
+      <c r="H38" t="s">
+        <v>222</v>
+      </c>
+      <c r="I38" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>224</v>
+      </c>
+      <c r="B39" t="s">
+        <v>225</v>
+      </c>
+      <c r="C39" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" t="s">
+        <v>226</v>
+      </c>
+      <c r="E39" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" t="s">
+        <v>45</v>
+      </c>
+      <c r="G39" t="s">
+        <v>227</v>
+      </c>
+      <c r="H39" t="s">
+        <v>228</v>
+      </c>
+      <c r="I39" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>230</v>
+      </c>
+      <c r="B40" t="s">
+        <v>231</v>
+      </c>
+      <c r="C40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" t="s">
+        <v>232</v>
+      </c>
+      <c r="E40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" t="s">
+        <v>45</v>
+      </c>
+      <c r="G40" t="s">
+        <v>233</v>
+      </c>
+      <c r="H40" t="s">
+        <v>234</v>
+      </c>
+      <c r="I40" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>236</v>
+      </c>
+      <c r="B41" t="s">
+        <v>237</v>
+      </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>238</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
+        <v>45</v>
+      </c>
+      <c r="G41" t="s">
+        <v>239</v>
+      </c>
+      <c r="H41" t="s">
+        <v>240</v>
+      </c>
+      <c r="I41" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>242</v>
+      </c>
+      <c r="B42" t="s">
+        <v>243</v>
+      </c>
+      <c r="C42" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" t="s">
+        <v>244</v>
+      </c>
+      <c r="E42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" t="s">
+        <v>27</v>
+      </c>
+      <c r="G42" t="s">
+        <v>245</v>
+      </c>
+      <c r="H42" t="s">
+        <v>246</v>
+      </c>
+      <c r="I42" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>248</v>
+      </c>
+      <c r="B43" t="s">
+        <v>249</v>
+      </c>
+      <c r="C43" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" t="s">
+        <v>250</v>
+      </c>
+      <c r="E43" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" t="s">
+        <v>251</v>
+      </c>
+      <c r="G43" t="s">
+        <v>252</v>
+      </c>
+      <c r="H43" t="s">
+        <v>253</v>
+      </c>
+      <c r="I43" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>255</v>
+      </c>
+      <c r="B44" t="s">
+        <v>256</v>
+      </c>
+      <c r="C44" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" t="s">
+        <v>257</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
+        <v>45</v>
+      </c>
+      <c r="G44" t="s">
+        <v>258</v>
+      </c>
+      <c r="H44" t="s">
+        <v>259</v>
+      </c>
+      <c r="I44" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>261</v>
+      </c>
+      <c r="B45" t="s">
+        <v>262</v>
+      </c>
+      <c r="C45" t="s">
+        <v>263</v>
+      </c>
+      <c r="D45" t="s">
+        <v>264</v>
+      </c>
+      <c r="E45" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" t="s">
+        <v>45</v>
+      </c>
+      <c r="G45" t="s">
+        <v>265</v>
+      </c>
+      <c r="H45" t="s">
+        <v>47</v>
+      </c>
+      <c r="I45" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>267</v>
+      </c>
+      <c r="B46" t="s">
+        <v>268</v>
+      </c>
+      <c r="C46" t="s">
+        <v>269</v>
+      </c>
+      <c r="D46" t="s">
+        <v>270</v>
+      </c>
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" t="s">
+        <v>45</v>
+      </c>
+      <c r="G46" t="s">
+        <v>271</v>
+      </c>
+      <c r="H46" t="s">
+        <v>47</v>
+      </c>
+      <c r="I46" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>273</v>
+      </c>
+      <c r="B47" t="s">
+        <v>249</v>
+      </c>
+      <c r="C47" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" t="s">
+        <v>274</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
+        <v>251</v>
+      </c>
+      <c r="G47" t="s">
+        <v>275</v>
+      </c>
+      <c r="H47" t="s">
+        <v>253</v>
+      </c>
+      <c r="I47" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>277</v>
+      </c>
+      <c r="B48" t="s">
+        <v>278</v>
+      </c>
+      <c r="C48" t="s">
+        <v>279</v>
+      </c>
+      <c r="D48" t="s">
+        <v>280</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
+        <v>21</v>
+      </c>
+      <c r="G48" t="s">
+        <v>281</v>
+      </c>
+      <c r="H48" t="s">
+        <v>172</v>
+      </c>
+      <c r="I48" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>283</v>
+      </c>
+      <c r="B49" t="s">
+        <v>284</v>
+      </c>
+      <c r="C49" t="s">
+        <v>285</v>
+      </c>
+      <c r="D49" t="s">
+        <v>286</v>
+      </c>
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
+        <v>21</v>
+      </c>
+      <c r="G49" t="s">
+        <v>287</v>
+      </c>
+      <c r="H49" t="s">
+        <v>172</v>
+      </c>
+      <c r="I49" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>289</v>
+      </c>
+      <c r="B50" t="s">
+        <v>268</v>
+      </c>
+      <c r="C50" t="s">
+        <v>290</v>
+      </c>
+      <c r="D50" t="s">
+        <v>291</v>
+      </c>
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" t="s">
+        <v>292</v>
+      </c>
+      <c r="H50" t="s">
+        <v>172</v>
+      </c>
+      <c r="I50" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>294</v>
+      </c>
+      <c r="B51" t="s">
+        <v>278</v>
+      </c>
+      <c r="C51" t="s">
+        <v>295</v>
+      </c>
+      <c r="D51" t="s">
+        <v>296</v>
+      </c>
+      <c r="E51" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" t="s">
+        <v>297</v>
+      </c>
+      <c r="H51" t="s">
+        <v>172</v>
+      </c>
+      <c r="I51" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>299</v>
+      </c>
+      <c r="B52" t="s">
+        <v>268</v>
+      </c>
+      <c r="C52" t="s">
+        <v>300</v>
+      </c>
+      <c r="D52" t="s">
+        <v>301</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" t="s">
+        <v>302</v>
+      </c>
+      <c r="H52" t="s">
+        <v>172</v>
+      </c>
+      <c r="I52" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>304</v>
+      </c>
+      <c r="B53" t="s">
+        <v>268</v>
+      </c>
+      <c r="C53" t="s">
+        <v>305</v>
+      </c>
+      <c r="D53" t="s">
+        <v>306</v>
+      </c>
+      <c r="E53" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" t="s">
+        <v>307</v>
+      </c>
+      <c r="H53" t="s">
+        <v>172</v>
+      </c>
+      <c r="I53" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>309</v>
+      </c>
+      <c r="B54" t="s">
+        <v>268</v>
+      </c>
+      <c r="C54" t="s">
+        <v>310</v>
+      </c>
+      <c r="D54" t="s">
+        <v>311</v>
+      </c>
+      <c r="E54" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" t="s">
+        <v>312</v>
+      </c>
+      <c r="H54" t="s">
+        <v>172</v>
+      </c>
+      <c r="I54" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>